<commit_message>
Add uncertainty.py and update Excel
Introduce uncertainty.py: a script that computes alpha-energy means, counting uncertainty (from FWHM), total uncertainty, and the implied calibration uncertainty (ΔEcal) needed to reproduce reported uncertainties. It compares listed-event means against reported results for two decay chains and prints a concise summary. Also updates Calc_Gamma_Recoil_Correction.xlsx (binary changes).
</commit_message>
<xml_diff>
--- a/Calc_Gamma_Recoil_Correction.xlsx
+++ b/Calc_Gamma_Recoil_Correction.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Si24\root_scripts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCDCFCCD-6621-44BF-9A65-49813F7F6519}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{553FBD57-83C0-4188-B0B9-D3CD53E2EE1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7896" yWindow="36" windowWidth="15144" windowHeight="12000" xr2:uid="{9BE0492A-2FA3-4C66-B5FA-754BC23C79FC}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" xr2:uid="{9BE0492A-2FA3-4C66-B5FA-754BC23C79FC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -28,6 +28,9 @@
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -177,10 +180,10 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -598,7 +601,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="10" t="s">
         <v>10</v>
       </c>
     </row>
@@ -618,7 +621,7 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="3">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
@@ -647,11 +650,11 @@
       </c>
       <c r="B5" s="6">
         <f>E5*1000</f>
-        <v>3.7910501774636826E-2</v>
+        <v>3.9025516532714383E-2</v>
       </c>
       <c r="C5" s="4">
         <f>A5+B5</f>
-        <v>1572.2779105017746</v>
+        <v>1572.2790255165328</v>
       </c>
       <c r="D5" s="1">
         <f>A5/1000</f>
@@ -659,11 +662,11 @@
       </c>
       <c r="E5" s="7">
         <f>D5^2/2/$A$3/$D$2</f>
-        <v>3.791050177463683E-5</v>
+        <v>3.902551653271438E-5</v>
       </c>
       <c r="F5" s="9">
         <f>C5/1000</f>
-        <v>1.5722779105017746</v>
+        <v>1.5722790255165329</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
@@ -687,28 +690,28 @@
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="10">
+      <c r="A8" s="11">
         <f>C8-B8</f>
-        <v>2347.4154851446924</v>
+        <v>3128.8454311043602</v>
       </c>
       <c r="B8" s="6">
         <f>E8*1000</f>
-        <v>8.4514855307390932E-2</v>
+        <v>0.15456889563962417</v>
       </c>
       <c r="C8" s="8">
-        <v>2347.5</v>
+        <v>3129</v>
       </c>
       <c r="D8" s="9">
         <f>A8/1000</f>
-        <v>2.3474154851446922</v>
+        <v>3.1288454311043603</v>
       </c>
       <c r="E8" s="7">
         <f>F8^2/2/$A$3/$D$2</f>
-        <v>8.4514855307390936E-5</v>
+        <v>1.5456889563962418E-4</v>
       </c>
       <c r="F8" s="9">
         <f>C8/1000</f>
-        <v>2.3475000000000001</v>
+        <v>3.129</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Add Calc_Width_Lifetime.py for decay width calculation
</commit_message>
<xml_diff>
--- a/Calc_Gamma_Recoil_Correction.xlsx
+++ b/Calc_Gamma_Recoil_Correction.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Si24\root_scripts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{553FBD57-83C0-4188-B0B9-D3CD53E2EE1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63624FA8-6F9F-466B-BA83-DF103B775D86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" xr2:uid="{9BE0492A-2FA3-4C66-B5FA-754BC23C79FC}"/>
   </bookViews>
@@ -646,27 +646,27 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="3">
-        <v>1572.24</v>
+        <v>3305</v>
       </c>
       <c r="B5" s="6">
         <f>E5*1000</f>
-        <v>3.9025516532714383E-2</v>
+        <v>0.17244630982731424</v>
       </c>
       <c r="C5" s="4">
         <f>A5+B5</f>
-        <v>1572.2790255165328</v>
+        <v>3305.1724463098271</v>
       </c>
       <c r="D5" s="1">
         <f>A5/1000</f>
-        <v>1.5722400000000001</v>
+        <v>3.3050000000000002</v>
       </c>
       <c r="E5" s="7">
         <f>D5^2/2/$A$3/$D$2</f>
-        <v>3.902551653271438E-5</v>
+        <v>1.7244630982731423E-4</v>
       </c>
       <c r="F5" s="9">
         <f>C5/1000</f>
-        <v>1.5722790255165329</v>
+        <v>3.3051724463098271</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Update half-life values in Calc_Width_Lifetime.py for decay width calculation
</commit_message>
<xml_diff>
--- a/Calc_Gamma_Recoil_Correction.xlsx
+++ b/Calc_Gamma_Recoil_Correction.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Si24\root_scripts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63624FA8-6F9F-466B-BA83-DF103B775D86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{649A473C-66E7-44B4-94D9-193C91BD0D71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" xr2:uid="{9BE0492A-2FA3-4C66-B5FA-754BC23C79FC}"/>
+    <workbookView xWindow="5760" yWindow="0" windowWidth="17280" windowHeight="9072" xr2:uid="{9BE0492A-2FA3-4C66-B5FA-754BC23C79FC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -621,7 +621,7 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="3">
-        <v>34</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
@@ -646,27 +646,27 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="3">
-        <v>3305</v>
+        <v>7333</v>
       </c>
       <c r="B5" s="6">
         <f>E5*1000</f>
-        <v>0.17244630982731424</v>
+        <v>1.2549471271896568</v>
       </c>
       <c r="C5" s="4">
         <f>A5+B5</f>
-        <v>3305.1724463098271</v>
+        <v>7334.2549471271896</v>
       </c>
       <c r="D5" s="1">
         <f>A5/1000</f>
-        <v>3.3050000000000002</v>
+        <v>7.3330000000000002</v>
       </c>
       <c r="E5" s="7">
         <f>D5^2/2/$A$3/$D$2</f>
-        <v>1.7244630982731423E-4</v>
+        <v>1.2549471271896568E-3</v>
       </c>
       <c r="F5" s="9">
         <f>C5/1000</f>
-        <v>3.3051724463098271</v>
+        <v>7.3342549471271896</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
@@ -692,22 +692,22 @@
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="11">
         <f>C8-B8</f>
-        <v>3128.8454311043602</v>
+        <v>3128.7715068499242</v>
       </c>
       <c r="B8" s="6">
         <f>E8*1000</f>
-        <v>0.15456889563962417</v>
+        <v>0.22849315007596616</v>
       </c>
       <c r="C8" s="8">
         <v>3129</v>
       </c>
       <c r="D8" s="9">
         <f>A8/1000</f>
-        <v>3.1288454311043603</v>
+        <v>3.1287715068499242</v>
       </c>
       <c r="E8" s="7">
         <f>F8^2/2/$A$3/$D$2</f>
-        <v>1.5456889563962418E-4</v>
+        <v>2.2849315007596616E-4</v>
       </c>
       <c r="F8" s="9">
         <f>C8/1000</f>

</xml_diff>